<commit_message>
TS 2.4 Kramam files corrections
</commit_message>
<xml_diff>
--- a/TS Jatai Working/TTD Krama PaarayaNam.xlsx
+++ b/TS Jatai Working/TTD Krama PaarayaNam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\texts\TS Jatai Working\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01532C57-83B0-48BB-B5EB-88A463EB2CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kandam1 to 7" sheetId="1" r:id="rId1"/>
@@ -1959,7 +1959,7 @@
     <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="72" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>

</xml_diff>